<commit_message>
Lisans sistemi geri getirildi: lisans.py git gecmisinden kurtarildi, app_portal.py/portal_watchdog.py'a yeniden baglandi. Sablona Makine ID alani ve otomasyona Supabase lisanlar tablosu kaydi eklendi
</commit_message>
<xml_diff>
--- a/yeni_lokasyon_kurulum_sablonu.xlsx
+++ b/yeni_lokasyon_kurulum_sablonu.xlsx
@@ -629,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1344,13 +1344,40 @@
         </is>
       </c>
     </row>
+    <row r="51" ht="8" customHeight="1"/>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7. LiSANS BiLGiSi (Lokasyon ID ile KARISTIRMAYIN — farkli kavramlar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Makine ID</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Lokasyon PC sinin anakart UUID si — PC de "wmic csproduct get uuid" komutuyla alinir. Bu, Lokasyon ID DEGiLDiR, ayri bir kavramdir.</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Ornek: DF9ABA0D-A7A8-C416-A430-00D861BD5794</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A52:D52"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A11:D11"/>

</xml_diff>

<commit_message>
Lokasyon kurulum sablonu SAGLAMLASTIRMA'ya gore guncellendi (8/8 test) - lokasyon_kurulum_otomasyon.py: _ahu_nokta_tipi collector _detect_point_type ile birebir senkron (Start/Stop + Basinc taninir, taninmayan ad Return VARSAYILMAZ -> bos doner + kurulumda uyari); ahu_noktalari_oku tanimlanamayan noktayi atlar - hvac_settings_uret: SAT_HEATING varsayilan 27/30 -> 28/31; on kosul kapisi esikleri eklendi (PRESSURE_RUN_MIN_PA, PRESSURE_FAULT_MAX_PA, SENSOR_VALID_MIN/MAX_C, MANUAL_SUPPRESS_HOURS, DEBOUNCE/DUZELME/TAKILI/ESKALASYON) -> yeni lokasyon config'i main_portal fail-fast'ten temiz gecer, on_kosul degerleri CONFIG'ten override alir - create_lokasyon_sablonu.py (Excel uretici): AHU Noktalari sayfasi Start/Basinc nokta tiplerini + Object Type bilgisini aciklar, taninmayan-ad-atlanir uyarisi; Isitma ufleme bandi varsayilan 28/31; Talimatlar'a ON KOSUL KAPISI acikamasi eklendi - yeni_lokasyon_kurulum_sablonu.xlsx yeniden uretildi
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yeni_lokasyon_kurulum_sablonu.xlsx
+++ b/yeni_lokasyon_kurulum_sablonu.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -123,6 +123,12 @@
       <color rgb="00833C00"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -184,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -263,6 +269,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1183,12 +1192,12 @@
       <c r="B40" s="5" t="n"/>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Bos = varsayilan 27.0 kullanilir</t>
+          <t>Bos = varsayilan 28.0 kullanilir</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Ornek: 27.0</t>
+          <t>Ornek: 28.0</t>
         </is>
       </c>
     </row>
@@ -1201,12 +1210,12 @@
       <c r="B41" s="5" t="n"/>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Bos = varsayilan 30.0 kullanilir</t>
+          <t>Bos = varsayilan 31.0 kullanilir</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Ornek: 30.0</t>
+          <t>Ornek: 31.0</t>
         </is>
       </c>
     </row>
@@ -2452,10 +2461,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Bu sayfa SANTRAL (chiller/kazan) noktalarindan AYRIDIR — sadece AHU (klima santrali) noktalari icin kullanilir. ahu_collector.py --setup ile islenir.</t>
+          <t>Bu sayfa SANTRAL (chiller/kazan) noktalarindan AYRIDIR — sadece AHU (klima santrali) noktalari icin kullanilir. ahu_collector.py --setup ile islenir.  YENI: Her AHU icin sicaklik/vana noktalarina EK OLARAK "Start/Stop" (calisma komutu, binary Object Type=4) ve "Basinc" (kanal fark basinci Pa, analog Object Type=0) noktalari da girilebilir — bunlar ON KOSUL KAPISI icin kullanilir (santral gercekten calisiyor mu, fan basiyor mu, sensor saglam mi). Basinc sensoru olmayan santrallerde basinc noktasi bos birakilir (kapi otomatik 2/3 onaya duser).</t>
         </is>
       </c>
     </row>
@@ -3035,10 +3044,10 @@
       <c r="G54" s="5" t="n"/>
       <c r="H54" s="5" t="n"/>
     </row>
-    <row r="55" ht="54" customHeight="1">
+    <row r="55" ht="78" customHeight="1">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>ONEMLI — Point Name formati: ILK KELIME AHU adidir (orn. "Ahu-3"), sistem bunu otomatik ayirir. Devamindaki kelimeye gore nokta tipi otomatik tespit edilir: "Ufleme" iceren -&gt; SAT/ufleme sicakligi  |  "...Sogutma Vana..." -&gt; sogutma vana yuzdesi  |  "...Isitma Vana..." -&gt; isitma vana yuzdesi  |  "...Set" ile bitenler -&gt; set sicakligi  |  digerleri -&gt; emis/donus sicakligi. Ornekler: "Ahu-3 Ufleme", "Ahu-3 Emis", "Ahu-3 Isitma Vana", "Ahu-3 Sogutma Vana", "Ahu-3 Set". LOCATION (MAHAL) sutunu hangi hat/bolgede oldugunu belirtir (orn. MAS-1, MAS-2 — Lokasyon Profili sayfasindaki Hat 1/Hat 2 adlarina karsilik gelir).</t>
+          <t>ONEMLI — Point Name formati: ILK KELIME AHU adidir (orn. "Ahu-3"), sistem bunu otomatik ayirir. Devamindaki kelimeye gore nokta tipi otomatik tespit edilir: "Start" iceren -&gt; Start/Stop komutu (Object Type=4)  |  "Basinc" iceren -&gt; kanal basinci Pa (Object Type=0)  |  "Ufleme" iceren -&gt; SAT/ufleme sicakligi  |  "...Sogutma Vana..." -&gt; sogutma vana yuzdesi  |  "...Isitma Vana..." -&gt; isitma vana yuzdesi  |  "...Set" ile bitenler -&gt; set sicakligi  |  "Emis/Donus" iceren -&gt; emis/donus sicakligi. Ornekler: "Ahu-3 Ufleme", "Ahu-3 Emis", "Ahu-3 Isitma Vana", "Ahu-3 Sogutma Vana", "Ahu-3 Set", "Ahu-3 Start", "Ahu-3 Basinc". DIKKAT: Bu anahtar kelimelerden HICBIRINI icermeyen isimler ARTIK atlanir (eskiden yanlislikla emis sayiliyordu) — tanimlanamayan nokta konfige eklenmez, kurulumda uyari verilir. LOCATION (MAHAL): hangi hat/bolge (orn. MAS-1, MAS-2 — Lokasyon Profili Hat 1/Hat 2 adlarina karsilik).</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3421,7 +3430,7 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>AHU Noktalari sayfasina klima santrali (AHU) noktalarini girin — santral noktalarindan AYRI sayfa</t>
+          <t>AHU Noktalari sayfasina klima santrali (AHU) noktalarini girin — santral noktalarindan AYRI sayfa. Sicaklik/vana noktalarina EK OLARAK varsa "Ahu-X Start" (Object Type=4) ve "Ahu-X Basinc" (Object Type=0) noktalarini da girin — on kosul kapisi bunlari kullanir</t>
         </is>
       </c>
     </row>
@@ -3497,7 +3506,7 @@
       <c r="A14" s="21" t="inlineStr"/>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - hvac_settings.json  (Genel AHU Ufleme Bandi alanlarindan, CONFIG override — kaynak kod degismez)</t>
+          <t xml:space="preserve">  - hvac_settings.json  (Genel AHU Ufleme Bandi + on kosul kapisi esikleri: basinc/sensor gecerlilik araliklari, susturma suresi vb. — CONFIG override, kaynak kod degismez)</t>
         </is>
       </c>
     </row>
@@ -3654,6 +3663,18 @@
       <c r="B31" s="26" t="inlineStr">
         <is>
           <t>Veri Okuma Saati / GM Sync Saati alanlari bilgi amaclidir, sistemde sabittir (07:10 / 08:00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="58" customHeight="1">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>YENI</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>ON KOSUL KAPISI: AHU Start/Basinc noktalari girilirse, analiz oncesi 3 kapili kontrol calisir (1-santral calisiyor mu, 2-fan basinc uretiyor mu, 3-sensorler saglam mi). Kapiyi gecemeyen santral "Analiz Disi" isaretlenir, sahte alarm uretilmez. Basinc noktasi olmayan santral 2/3 onayla analiz edilir. Start/Basinc noktalari YOKSA eski davranis aynen surer (kapi devreye girmez).</t>
         </is>
       </c>
     </row>

</xml_diff>